<commit_message>
api test is ok
</commit_message>
<xml_diff>
--- a/J3270-API.xlsx
+++ b/J3270-API.xlsx
@@ -5,16 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\tmp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\03_src\tn3270-api-project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB00729-86B4-4F61-A167-F738A2B0718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD2E9B7-5C70-4C58-8B5D-8CA968771B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17430" yWindow="570" windowWidth="27165" windowHeight="14640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14085" yWindow="1020" windowWidth="33000" windowHeight="14190" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="API" sheetId="1" r:id="rId1"/>
-    <sheet name="flow" sheetId="2" r:id="rId2"/>
+    <sheet name="API_list" sheetId="1" r:id="rId1"/>
+    <sheet name="backendざっくり検証" sheetId="2" r:id="rId2"/>
+    <sheet name="frontendざっくり動作確認" sheetId="3" r:id="rId3"/>
+    <sheet name="backend_logo" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t>### 2. API1: 登录到 TSO 主菜单</t>
   </si>
@@ -88,6 +90,222 @@
   <si>
     <t>### 在当前位置输入字符串</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>D:\Program_Files\jdks\corretto-21.0.9\bin\java.exe -XX:TieredStopAtLevel=1 -Dspring.output.ansi.enabled=always -Dcom.sun.management.jmxremote -Dspring.jmx.enabled=true -Dspring.liveBeansView.mbeanDomain -Dspring.application.admin.enabled=true "-Dmanagement.endpoints.jmx.exposure.include=*" -javaagent:D:\ideaIU-2024.3.win\lib\idea_rt.jar=10050:D:\ideaIU-2024.3.win\bin -Dfile.encoding=UTF-8 -Dsun.stdout.encoding=UTF-8 -Dsun.stderr.encoding=UTF-8 -classpath E:\03_src\tn3270-api-project\target\classes;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-starter-web\4.0.0\spring-boot-starter-web-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-starter-jackson\4.0.0\spring-boot-starter-jackson-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-jackson\4.0.0\spring-boot-jackson-4.0.0.jar;C:\Users\bieyu\.m2\repository\tools\jackson\core\jackson-databind\3.0.2\jackson-databind-3.0.2.jar;C:\Users\bieyu\.m2\repository\com\fasterxml\jackson\core\jackson-annotations\2.20\jackson-annotations-2.20.jar;C:\Users\bieyu\.m2\repository\tools\jackson\core\jackson-core\3.0.2\jackson-core-3.0.2.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-starter-tomcat\4.0.0\spring-boot-starter-tomcat-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-starter-tomcat-runtime\4.0.0\spring-boot-starter-tomcat-runtime-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-web-server\4.0.0\spring-boot-web-server-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\apache\tomcat\embed\tomcat-embed-core\11.0.14\tomcat-embed-core-11.0.14.jar;C:\Users\bieyu\.m2\repository\org\apache\tomcat\embed\tomcat-embed-el\11.0.14\tomcat-embed-el-11.0.14.jar;C:\Users\bieyu\.m2\repository\org\apache\tomcat\embed\tomcat-embed-websocket\11.0.14\tomcat-embed-websocket-11.0.14.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-tomcat\4.0.0\spring-boot-tomcat-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-http-converter\4.0.0\spring-boot-http-converter-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot\4.0.0\spring-boot-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\spring-context\7.0.1\spring-context-7.0.1.jar;C:\Users\bieyu\.m2\repository\org\springframework\spring-web\7.0.1\spring-web-7.0.1.jar;C:\Users\bieyu\.m2\repository\org\springframework\spring-beans\7.0.1\spring-beans-7.0.1.jar;C:\Users\bieyu\.m2\repository\io\micrometer\micrometer-observation\1.16.0\micrometer-observation-1.16.0.jar;C:\Users\bieyu\.m2\repository\io\micrometer\micrometer-commons\1.16.0\micrometer-commons-1.16.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-webmvc\4.0.0\spring-boot-webmvc-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-servlet\4.0.0\spring-boot-servlet-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\spring-webmvc\7.0.1\spring-webmvc-7.0.1.jar;C:\Users\bieyu\.m2\repository\org\springframework\spring-aop\7.0.1\spring-aop-7.0.1.jar;C:\Users\bieyu\.m2\repository\org\springframework\spring-expression\7.0.1\spring-expression-7.0.1.jar;C:\Users\bieyu\.m2\repository\org\projectlombok\lombok\1.18.42\lombok-1.18.42.jar;C:\Users\bieyu\.m2\repository\com\github\filipesimoes\j3270\1.0.2\j3270-1.0.2.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-starter\4.0.0\spring-boot-starter-4.0.0.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-starter-logging\4.0.0\spring-boot-starter-logging-4.0.0.jar;C:\Users\bieyu\.m2\repository\ch\qos\logback\logback-classic\1.5.21\logback-classic-1.5.21.jar;C:\Users\bieyu\.m2\repository\ch\qos\logback\logback-core\1.5.21\logback-core-1.5.21.jar;C:\Users\bieyu\.m2\repository\org\apache\logging\log4j\log4j-to-slf4j\2.25.2\log4j-to-slf4j-2.25.2.jar;C:\Users\bieyu\.m2\repository\org\apache\logging\log4j\log4j-api\2.25.2\log4j-api-2.25.2.jar;C:\Users\bieyu\.m2\repository\org\slf4j\jul-to-slf4j\2.0.17\jul-to-slf4j-2.0.17.jar;C:\Users\bieyu\.m2\repository\org\springframework\boot\spring-boot-autoconfigure\4.0.0\spring-boot-autoconfigure-4.0.0.jar;C:\Users\bieyu\.m2\repository\jakarta\annotation\jakarta.annotation-api\3.0.0\jakarta.annotation-api-3.0.0.jar;C:\Users\bieyu\.m2\repository\org\yaml\snakeyaml\2.5\snakeyaml-2.5.jar;C:\Users\bieyu\.m2\repository\org\slf4j\slf4j-api\2.0.17\slf4j-api-2.0.17.jar;C:\Users\bieyu\.m2\repository\org\springframework\spring-core\7.0.1\spring-core-7.0.1.jar;C:\Users\bieyu\.m2\repository\commons-logging\commons-logging\1.3.5\commons-logging-1.3.5.jar;C:\Users\bieyu\.m2\repository\org\jspecify\jspecify\1.0.0\jspecify-1.0.0.jar com.example.tn3270api.Tn3270ApiApplication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  .   ____          _            __ _ _</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> /\\ / ___'_ __ _ _(_)_ __  __ _ \ \ \ \</t>
+  </si>
+  <si>
+    <t>( ( )\___ | '_ | '_| | '_ \/ _` | \ \ \ \</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> \\/  ___)| |_)| | | | | || (_| |  ) ) ) )</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  '  |____| .__|_| |_|_| |_\__, | / / / /</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =========|_|==============|___/=/_/_/_/</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> :: Spring Boot ::                (v4.0.0)</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.187 [main] INFO  c.e.tn3270api.Tn3270ApiApplication - Starting Tn3270ApiApplication using Java 21.0.9 with PID 34284 (E:\03_src\tn3270-api-project\target\classes started by bieyu in E:\03_src\tn3270-api-project)</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.189 [main] DEBUG c.e.tn3270api.Tn3270ApiApplication - Running with Spring Boot v4.0.0, Spring v7.0.1</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.190 [main] INFO  c.e.tn3270api.Tn3270ApiApplication - No active profile set, falling back to 1 default profile: "default"</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.637 [main] INFO  o.s.boot.tomcat.TomcatWebServer - Tomcat initialized with port 8080 (http)</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.648 [main] INFO  o.a.catalina.core.StandardService - Starting service [Tomcat]</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.649 [main] INFO  o.a.catalina.core.StandardEngine - Starting Servlet engine: [Apache Tomcat/11.0.14]</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.672 [main] INFO  o.s.b.w.c.s.WebApplicationContextInitializer - Root WebApplicationContext: initialization completed in 454 ms</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.862 [main] INFO  o.s.boot.tomcat.TomcatWebServer - Tomcat started on port 8080 (http) with context path '/'</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:34:57.864 [main] INFO  c.e.tn3270api.Tn3270ApiApplication - Started Tn3270ApiApplication in 0.983 seconds (process running for 1.383)</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:43.026 [http-nio-8080-exec-1] INFO  o.a.c.c.C.[Tomcat].[localhost].[/] - Initializing Spring DispatcherServlet 'dispatcherServlet'</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:43.026 [http-nio-8080-exec-1] INFO  o.s.web.servlet.DispatcherServlet - Initializing Servlet 'dispatcherServlet'</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:43.027 [http-nio-8080-exec-1] INFO  o.s.web.servlet.DispatcherServlet - Completed initialization in 0 ms</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:43.065 [http-nio-8080-exec-2] INFO  c.e.t.controller.Tn3270Controller - 收到登录请求</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:43.066 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 创建新会话: ab89cac8-fd4b-467c-83ff-cb0e25267d20</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:43.067 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 启动 3270 模拟器...</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:46.191 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 连接到主机: 127.0.0.1:3270</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:46.194 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 连接成功，等待主机响应...</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:46.194 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 等待键盘解锁...</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:51.401 [http-nio-8080-exec-2] WARN  c.e.tn3270api.service.Tn3270Service - 未找到 LOGON 文字，执行 CLEAR 和 RESET...</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:53.410 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 开始登录流程...</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:53.410 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 输入用户名: HERC01</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:35:54.427 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 提交用户名</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:36:01.449 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 输入密码</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:36:02.452 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 提交密码</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:36:05.463 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 提交登录信息</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:36:08.467 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 进入主菜单</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:36:10.479 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 登录成功，会话已保存: ab89cac8-fd4b-467c-83ff-cb0e25267d20</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:36:10.682 [http-nio-8080-exec-2] INFO  c.e.t.controller.Tn3270Controller - 登录成功，会话ID: ab89cac8-fd4b-467c-83ff-cb0e25267d20</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:38:46.948 [http-nio-8080-exec-5] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送字符串: X</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:38:46.948 [http-nio-8080-exec-5] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 在当前光标位置输入字符串: X</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:38:48.683 [http-nio-8080-exec-7] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:38:48.683 [http-nio-8080-exec-7] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:38:53.410 [http-nio-8080-exec-9] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 获取屏幕内容</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:39:09.941 [http-nio-8080-exec-10] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 获取屏幕内容</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:39:30.277 [http-nio-8080-exec-1] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送字符串: X</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:39:30.277 [http-nio-8080-exec-1] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 在当前光标位置输入字符串: X</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:39:31.994 [http-nio-8080-exec-2] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:39:31.994 [http-nio-8080-exec-2] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:39:36.715 [http-nio-8080-exec-3] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 获取屏幕内容</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:10.972 [http-nio-8080-exec-4] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送字符串: TSOAPPLS</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:10.972 [http-nio-8080-exec-4] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 在当前光标位置输入字符串: TSOAPPLS</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:12.696 [http-nio-8080-exec-5] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:12.696 [http-nio-8080-exec-5] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:17.428 [http-nio-8080-exec-6] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 获取屏幕内容</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:56.478 [http-nio-8080-exec-7] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送字符串: 2</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:56.478 [http-nio-8080-exec-7] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 在当前光标位置输入字符串: 2</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:58.195 [http-nio-8080-exec-8] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:40:58.195 [http-nio-8080-exec-8] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:02.918 [http-nio-8080-exec-9] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 获取屏幕内容</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:26.088 [http-nio-8080-exec-10] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送字符串: X</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:26.088 [http-nio-8080-exec-10] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 在当前光标位置输入字符串: X</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:27.806 [http-nio-8080-exec-1] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:27.806 [http-nio-8080-exec-1] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:32.531 [http-nio-8080-exec-2] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 获取屏幕内容</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:57.005 [http-nio-8080-exec-3] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送字符串: X</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:57.005 [http-nio-8080-exec-3] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 在当前光标位置输入字符串: X</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:58.726 [http-nio-8080-exec-4] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:41:58.726 [http-nio-8080-exec-4] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:42:03.443 [http-nio-8080-exec-5] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 获取屏幕内容</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:43:55.239 [http-nio-8080-exec-7] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送字符串: LOGOFF</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:43:55.239 [http-nio-8080-exec-7] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 在当前光标位置输入字符串: LOGOFF</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:43:56.968 [http-nio-8080-exec-8] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:43:56.968 [http-nio-8080-exec-8] INFO  c.e.tn3270api.service.Tn3270Service - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 发送回车键</t>
+  </si>
+  <si>
+    <t>2025-11-26 15:44:01.714 [http-nio-8080-exec-9] INFO  c.e.t.controller.Tn3270Controller - 会话 ab89cac8-fd4b-467c-83ff-cb0e25267d20 获取屏幕内容</t>
   </si>
 </sst>
 </file>
@@ -1151,6 +1369,583 @@
         <a:xfrm>
           <a:off x="5076825" y="18630900"/>
           <a:ext cx="9211961" cy="5944430"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>3155</xdr:colOff>
+      <xdr:row>76</xdr:row>
+      <xdr:rowOff>78126</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="图片 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFAF0F66-999D-7C81-F411-C5EBEBBBC67B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="714375" y="28575"/>
+          <a:ext cx="22605980" cy="13803651"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>241314</xdr:colOff>
+      <xdr:row>128</xdr:row>
+      <xdr:rowOff>115554</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="图片 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{653EE027-ACBA-AE10-869B-4725864F43A8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="704850" y="14297025"/>
+          <a:ext cx="22853664" cy="8983329"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>130</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>593777</xdr:colOff>
+      <xdr:row>188</xdr:row>
+      <xdr:rowOff>153862</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="图片 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BAAF1796-39F7-AE69-A168-81C97B7950F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="790575" y="23698200"/>
+          <a:ext cx="23120402" cy="10478962"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>250</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>422315</xdr:colOff>
+      <xdr:row>317</xdr:row>
+      <xdr:rowOff>58848</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="图片 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{76B2F088-BA45-4766-EBF9-A2F80D274A01}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="704850" y="34585275"/>
+          <a:ext cx="23034665" cy="12165123"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>320</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>441366</xdr:colOff>
+      <xdr:row>386</xdr:row>
+      <xdr:rowOff>135034</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="图片 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FCBBDDE2-7A68-006C-BFBB-C85C7AC92CC5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="714375" y="47244000"/>
+          <a:ext cx="23044191" cy="12069859"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>389</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>422312</xdr:colOff>
+      <xdr:row>465</xdr:row>
+      <xdr:rowOff>106707</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="图片 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CAB8483A-46F9-3AAC-ABB4-1D98726FB787}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="723900" y="59740800"/>
+          <a:ext cx="23015612" cy="13841757"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>468</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>546160</xdr:colOff>
+      <xdr:row>541</xdr:row>
+      <xdr:rowOff>173318</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="图片 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96FD2C07-3070-5E2A-6A9F-49336A631505}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="685800" y="74018775"/>
+          <a:ext cx="23177560" cy="13384493"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>544</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>527098</xdr:colOff>
+      <xdr:row>606</xdr:row>
+      <xdr:rowOff>163511</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="图片 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7BB361E-C3D0-566A-1D23-31E6DE5B477B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="752475" y="87791925"/>
+          <a:ext cx="23091823" cy="11364911"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>609</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>508048</xdr:colOff>
+      <xdr:row>686</xdr:row>
+      <xdr:rowOff>49575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="图片 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5FB3D486-FBF1-422A-61E6-02A2F34C2F79}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="733425" y="99545775"/>
+          <a:ext cx="23091823" cy="13975125"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>688</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>384207</xdr:colOff>
+      <xdr:row>748</xdr:row>
+      <xdr:rowOff>58664</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="图片 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E5A2F1F-1064-A61D-CD09-D04F5F719BD5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="723900" y="113899950"/>
+          <a:ext cx="22977507" cy="10850489"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>191</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>403262</xdr:colOff>
+      <xdr:row>246</xdr:row>
+      <xdr:rowOff>87124</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="图片 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D35F0568-CA85-45D5-8ADC-668423FBBCA2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="704850" y="34585275"/>
+          <a:ext cx="23015612" cy="10021699"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>750</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>336570</xdr:colOff>
+      <xdr:row>807</xdr:row>
+      <xdr:rowOff>96692</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="图片 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDAD4911-3782-9E21-2DF6-FB79CC8F143C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="762000" y="135807450"/>
+          <a:ext cx="22891770" cy="10336067"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>810</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>34</xdr:col>
+      <xdr:colOff>469945</xdr:colOff>
+      <xdr:row>871</xdr:row>
+      <xdr:rowOff>153959</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="图片 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DB1C8818-51D0-4E97-7DE6-0B3DCDCB6854}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="714375" y="146608800"/>
+          <a:ext cx="23072770" cy="11174384"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1426,94 +2221,94 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:B24"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
         <v>16</v>
       </c>
@@ -1527,10 +2322,392 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4428A61B-5248-4FE7-B82E-BF241E2F3AAE}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="13.9" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB931B5F-68E9-480A-AAC1-0D0B414496C5}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A995ADC4-15B5-4BD3-8123-2B2379223E47}">
+  <dimension ref="B3:B77"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B35" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B47" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B49" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B50" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B51" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B52" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B53" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B54" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B55" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B56" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B58" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B59" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B60" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B61" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B62" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B63" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B64" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B65" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B66" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B67" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="68" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B68" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="69" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B69" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="70" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B70" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="71" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B71" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="72" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B72" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="73" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B73" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="74" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B74" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="75" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B75" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="76" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B76" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="77" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B77" t="s">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>